<commit_message>
Added results for a-s3 MFDWC-GRL
</commit_message>
<xml_diff>
--- a/results/mfdwc_experiment_results.xlsx
+++ b/results/mfdwc_experiment_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\UDA-mfdwc-wavelet_features\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFC4D3D-8EC6-47EF-B95F-99B4FE792538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4064EC7-3331-40DA-B4FA-BBB4D6B44862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10890" xr2:uid="{207E8739-F5E8-4D4F-9227-D53A58B985A3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{207E8739-F5E8-4D4F-9227-D53A58B985A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -641,7 +641,7 @@
         <v>0.31819999999999998</v>
       </c>
       <c r="D8" s="2">
-        <v>0.3276</v>
+        <v>0.35749999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reorganize results: move plots, logs & checkpoints
Reorganize result artifacts: move many plot images and CSVs into results/plots/*, rename mfdwc-cnn outputs to results/mfdwc-baseline/*, and relocate csv_logs and model checkpoints accordingly. Remove obsolete files from results/archive/* and results/plots_mfdwc_baseline/; add new GRL plot assets and classification_report_s3.csv under results/plots/plots_mfdwc_grl/, and add training_time.txt for plots_mfdwc_cst. Also update the results/mfdwc_experiment_results.xlsx workbook. This cleans up and standardizes result directories for easier consumption.
</commit_message>
<xml_diff>
--- a/results/mfdwc_experiment_results.xlsx
+++ b/results/mfdwc_experiment_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\UDA-mfdwc-wavelet_features\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4064EC7-3331-40DA-B4FA-BBB4D6B44862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED112A5-8CBE-4944-BA62-9ACBB84A15BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{207E8739-F5E8-4D4F-9227-D53A58B985A3}"/>
+    <workbookView xWindow="7170" yWindow="2560" windowWidth="14400" windowHeight="7810" xr2:uid="{207E8739-F5E8-4D4F-9227-D53A58B985A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -641,7 +641,7 @@
         <v>0.31819999999999998</v>
       </c>
       <c r="D8" s="2">
-        <v>0.35749999999999998</v>
+        <v>0.35759999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>